<commit_message>
E-book Excel : chapitre 7 (5 projets en FCFA prouvés) et conclusion
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T8L22svZaEaGYSwza4q3Yc
</commit_message>
<xml_diff>
--- a/produits/preuves/sortie/c7-stock-piege/c7-stock-piege.xlsx
+++ b/produits/preuves/sortie/c7-stock-piege/c7-stock-piege.xlsx
@@ -294,7 +294,6 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="7.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="6.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="5.87"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -431,9 +430,6 @@
   </sheetPr>
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
-  <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="5.87"/>
-  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">

</xml_diff>